<commit_message>
Updated RT Data Pipeline
</commit_message>
<xml_diff>
--- a/0_0_Data/0_Forecast_Inputs/2_ifoCAST/ifoCAST_live_nowcast_series.xlsx
+++ b/0_0_Data/0_Forecast_Inputs/2_ifoCAST/ifoCAST_live_nowcast_series.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -578,6 +578,14 @@
         <v>0.042359665</v>
       </c>
     </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="2">
+        <v>46002</v>
+      </c>
+      <c r="B25">
+        <v>0.266698307</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>